<commit_message>
docs: add Domain C ERD, comprehensive ERD diagrams, data dictionary, and weekly plan
</commit_message>
<xml_diff>
--- a/tuan-02/Domain C/Data Dictionary domain C.xlsx
+++ b/tuan-02/Domain C/Data Dictionary domain C.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Iw1Z8zHvIdwFEYUDXFeZ0vsKDUtUtuxOTyYsXjH33Ik="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="YijPK6enQRXEYQV6rAY0Eob3+oCeKNNnyJj9x0zPWno="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="114">
   <si>
     <t>Bảng</t>
   </si>
@@ -231,13 +231,10 @@
     <t>sku_uom_conversions</t>
   </si>
   <si>
-    <t>Định danh quy tắc quy đổi</t>
-  </si>
-  <si>
     <t>sku_id</t>
   </si>
   <si>
-    <t>FK → skus.id, UK (with uom_id)</t>
+    <t>PK, FK → skus.id</t>
   </si>
   <si>
     <t>SKU áp dụng quy đổi</t>
@@ -246,7 +243,7 @@
     <t>uom_id</t>
   </si>
   <si>
-    <t>FK → uoms.id, UK (with sku_id)</t>
+    <t>PK, FK → uoms.id</t>
   </si>
   <si>
     <t>UOM cần quy đổi</t>
@@ -264,10 +261,13 @@
     <t>Định danh barcode</t>
   </si>
   <si>
-    <t>FK → skus.id</t>
+    <t>FK → sku_uom_conversions.sku_id</t>
   </si>
   <si>
     <t>SKU của barcode</t>
+  </si>
+  <si>
+    <t>FK → sku_uom_conversions.uom_id</t>
   </si>
   <si>
     <t>UOM tương ứng với barcode</t>
@@ -333,9 +333,6 @@
     <t>sku_suppliers</t>
   </si>
   <si>
-    <t>PK, FK → skus.id</t>
-  </si>
-  <si>
     <t>SKU được cung cấp</t>
   </si>
   <si>
@@ -367,7 +364,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -393,9 +390,13 @@
     <font>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
     <font/>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Times New Roman&quot;"/>
+    </font>
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -510,7 +511,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -546,7 +547,7 @@
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -554,8 +555,8 @@
     <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf borderId="1" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="3" numFmtId="22" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -568,6 +569,12 @@
     </xf>
     <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="3" numFmtId="22" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -593,10 +600,7 @@
     <xf borderId="1" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="5" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="8" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="3" numFmtId="22" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
@@ -820,7 +824,7 @@
     <col customWidth="1" min="3" max="3" width="18.88"/>
     <col customWidth="1" min="4" max="4" width="6.38"/>
     <col customWidth="1" min="5" max="5" width="13.38"/>
-    <col customWidth="1" min="6" max="6" width="24.88"/>
+    <col customWidth="1" min="6" max="6" width="32.75"/>
     <col customWidth="1" min="7" max="7" width="35.13"/>
     <col customWidth="1" min="8" max="8" width="15.25"/>
     <col customWidth="1" min="9" max="9" width="8.88"/>
@@ -1785,7 +1789,7 @@
         <v>70</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>11</v>
@@ -1794,14 +1798,14 @@
         <v>12</v>
       </c>
       <c r="E25" s="16"/>
-      <c r="F25" s="16" t="s">
-        <v>13</v>
+      <c r="F25" s="17" t="s">
+        <v>72</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H25" s="16">
-        <v>1.0</v>
+        <v>1001.0</v>
       </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
@@ -1825,7 +1829,7 @@
     <row r="26" ht="27.0" customHeight="1">
       <c r="A26" s="7"/>
       <c r="B26" s="15" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>11</v>
@@ -1835,13 +1839,13 @@
       </c>
       <c r="E26" s="16"/>
       <c r="F26" s="17" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H26" s="16">
-        <v>1001.0</v>
+        <v>2.0</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
@@ -1865,23 +1869,23 @@
     <row r="27" ht="27.0" customHeight="1">
       <c r="A27" s="7"/>
       <c r="B27" s="15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D27" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E27" s="16"/>
-      <c r="F27" s="17" t="s">
-        <v>76</v>
-      </c>
+      <c r="E27" s="16">
+        <v>1.0</v>
+      </c>
+      <c r="F27" s="16"/>
       <c r="G27" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H27" s="16">
-        <v>2.0</v>
+        <v>12.0</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
@@ -1905,23 +1909,21 @@
     <row r="28" ht="27.0" customHeight="1">
       <c r="A28" s="7"/>
       <c r="B28" s="15" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="D28" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E28" s="16">
-        <v>1.0</v>
-      </c>
+      <c r="E28" s="16"/>
       <c r="F28" s="16"/>
-      <c r="G28" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="H28" s="16">
-        <v>12.0</v>
+      <c r="G28" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="H28" s="18">
+        <v>46288.33333333334</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
@@ -1945,21 +1947,23 @@
     <row r="29" ht="27.0" customHeight="1">
       <c r="A29" s="7"/>
       <c r="B29" s="15" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D29" s="16" t="s">
         <v>12</v>
       </c>
       <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
+      <c r="F29" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G29" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="H29" s="18">
-        <v>46288.33333333334</v>
+        <v>53</v>
+      </c>
+      <c r="H29" s="16">
+        <v>101.0</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
@@ -1983,23 +1987,21 @@
     <row r="30" ht="27.0" customHeight="1">
       <c r="A30" s="7"/>
       <c r="B30" s="15" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="D30" s="16" t="s">
         <v>12</v>
       </c>
       <c r="E30" s="16"/>
-      <c r="F30" s="16" t="s">
-        <v>52</v>
-      </c>
+      <c r="F30" s="16"/>
       <c r="G30" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="H30" s="16">
-        <v>101.0</v>
+        <v>55</v>
+      </c>
+      <c r="H30" s="18">
+        <v>46288.375</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
@@ -2021,23 +2023,25 @@
       <c r="Z30" s="2"/>
     </row>
     <row r="31" ht="27.0" customHeight="1">
-      <c r="A31" s="7"/>
+      <c r="A31" s="9"/>
       <c r="B31" s="15" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D31" s="16" t="s">
         <v>12</v>
       </c>
       <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
+      <c r="F31" s="16" t="s">
+        <v>52</v>
+      </c>
       <c r="G31" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="H31" s="18">
-        <v>46288.375</v>
+        <v>57</v>
+      </c>
+      <c r="H31" s="16">
+        <v>101.0</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
@@ -2058,26 +2062,28 @@
       <c r="Y31" s="2"/>
       <c r="Z31" s="2"/>
     </row>
-    <row r="32" ht="27.0" customHeight="1">
-      <c r="A32" s="9"/>
-      <c r="B32" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="C32" s="16" t="s">
+    <row r="32" ht="13.5" customHeight="1">
+      <c r="A32" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="16" t="s">
+      <c r="D32" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="G32" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="H32" s="16">
-        <v>101.0</v>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="H32" s="21">
+        <v>1.0</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -2099,11 +2105,9 @@
       <c r="Z32" s="2"/>
     </row>
     <row r="33" ht="13.5" customHeight="1">
-      <c r="A33" s="19" t="s">
-        <v>80</v>
-      </c>
+      <c r="A33" s="7"/>
       <c r="B33" s="20" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="C33" s="21" t="s">
         <v>11</v>
@@ -2112,14 +2116,14 @@
         <v>12</v>
       </c>
       <c r="E33" s="21"/>
-      <c r="F33" s="21" t="s">
-        <v>13</v>
+      <c r="F33" s="22" t="s">
+        <v>81</v>
       </c>
       <c r="G33" s="21" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H33" s="21">
-        <v>1.0</v>
+        <v>1001.0</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
@@ -2143,7 +2147,7 @@
     <row r="34" ht="13.5" customHeight="1">
       <c r="A34" s="7"/>
       <c r="B34" s="20" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C34" s="21" t="s">
         <v>11</v>
@@ -2152,14 +2156,14 @@
         <v>12</v>
       </c>
       <c r="E34" s="21"/>
-      <c r="F34" s="21" t="s">
-        <v>82</v>
+      <c r="F34" s="23" t="s">
+        <v>83</v>
       </c>
       <c r="G34" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H34" s="21">
-        <v>1001.0</v>
+        <v>2.0</v>
       </c>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
@@ -2183,23 +2187,23 @@
     <row r="35" ht="13.5" customHeight="1">
       <c r="A35" s="7"/>
       <c r="B35" s="20" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="C35" s="21" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="D35" s="21" t="s">
         <v>12</v>
       </c>
       <c r="E35" s="21"/>
       <c r="F35" s="21" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G35" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="H35" s="21">
-        <v>2.0</v>
+        <v>86</v>
+      </c>
+      <c r="H35" s="20">
+        <v>8.938501234567E12</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -2223,23 +2227,21 @@
     <row r="36" ht="13.5" customHeight="1">
       <c r="A36" s="7"/>
       <c r="B36" s="20" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>29</v>
+        <v>88</v>
       </c>
       <c r="D36" s="21" t="s">
         <v>12</v>
       </c>
       <c r="E36" s="21"/>
-      <c r="F36" s="21" t="s">
-        <v>18</v>
-      </c>
+      <c r="F36" s="21"/>
       <c r="G36" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="H36" s="20">
-        <v>8.938501234567E12</v>
+        <v>89</v>
+      </c>
+      <c r="H36" s="20" t="s">
+        <v>90</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
@@ -2263,21 +2265,23 @@
     <row r="37" ht="13.5" customHeight="1">
       <c r="A37" s="7"/>
       <c r="B37" s="20" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>88</v>
+        <v>39</v>
       </c>
       <c r="D37" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="E37" s="21"/>
+      <c r="E37" s="20" t="b">
+        <v>0</v>
+      </c>
       <c r="F37" s="21"/>
       <c r="G37" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="H37" s="20" t="s">
-        <v>90</v>
+        <v>92</v>
+      </c>
+      <c r="H37" s="20" t="b">
+        <v>1</v>
       </c>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -2301,23 +2305,21 @@
     <row r="38" ht="13.5" customHeight="1">
       <c r="A38" s="7"/>
       <c r="B38" s="20" t="s">
-        <v>91</v>
+        <v>48</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="D38" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="E38" s="20" t="b">
-        <v>0</v>
-      </c>
+      <c r="E38" s="21"/>
       <c r="F38" s="21"/>
       <c r="G38" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="H38" s="20" t="b">
-        <v>1</v>
+        <v>50</v>
+      </c>
+      <c r="H38" s="24">
+        <v>46288.33333333334</v>
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
@@ -2341,21 +2343,23 @@
     <row r="39" ht="13.5" customHeight="1">
       <c r="A39" s="7"/>
       <c r="B39" s="20" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D39" s="21" t="s">
         <v>12</v>
       </c>
       <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
+      <c r="F39" s="21" t="s">
+        <v>52</v>
+      </c>
       <c r="G39" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="H39" s="22">
-        <v>46288.33333333334</v>
+        <v>53</v>
+      </c>
+      <c r="H39" s="21">
+        <v>101.0</v>
       </c>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
@@ -2379,23 +2383,21 @@
     <row r="40" ht="13.5" customHeight="1">
       <c r="A40" s="7"/>
       <c r="B40" s="20" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="D40" s="21" t="s">
         <v>12</v>
       </c>
       <c r="E40" s="21"/>
-      <c r="F40" s="21" t="s">
-        <v>52</v>
-      </c>
+      <c r="F40" s="21"/>
       <c r="G40" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="H40" s="21">
-        <v>101.0</v>
+        <v>55</v>
+      </c>
+      <c r="H40" s="24">
+        <v>46288.375</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
@@ -2417,23 +2419,25 @@
       <c r="Z40" s="2"/>
     </row>
     <row r="41" ht="13.5" customHeight="1">
-      <c r="A41" s="7"/>
+      <c r="A41" s="9"/>
       <c r="B41" s="20" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="D41" s="21" t="s">
         <v>12</v>
       </c>
       <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
+      <c r="F41" s="21" t="s">
+        <v>52</v>
+      </c>
       <c r="G41" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="H41" s="22">
-        <v>46288.375</v>
+        <v>57</v>
+      </c>
+      <c r="H41" s="21">
+        <v>101.0</v>
       </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
@@ -2455,25 +2459,27 @@
       <c r="Z41" s="2"/>
     </row>
     <row r="42" ht="13.5" customHeight="1">
-      <c r="A42" s="9"/>
-      <c r="B42" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="C42" s="21" t="s">
+      <c r="A42" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="B42" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="D42" s="21" t="s">
+      <c r="D42" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E42" s="21"/>
-      <c r="F42" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="G42" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="H42" s="21">
-        <v>101.0</v>
+      <c r="E42" s="27"/>
+      <c r="F42" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="H42" s="27">
+        <v>5001.0</v>
       </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
@@ -2495,27 +2501,25 @@
       <c r="Z42" s="2"/>
     </row>
     <row r="43" ht="13.5" customHeight="1">
-      <c r="A43" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="B43" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" s="25" t="s">
-        <v>11</v>
-      </c>
-      <c r="D43" s="25" t="s">
+      <c r="A43" s="7"/>
+      <c r="B43" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="C43" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D43" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E43" s="25"/>
-      <c r="F43" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="G43" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="H43" s="25">
-        <v>5001.0</v>
+      <c r="E43" s="27"/>
+      <c r="F43" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="G43" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="H43" s="26" t="s">
+        <v>96</v>
       </c>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
@@ -2538,24 +2542,22 @@
     </row>
     <row r="44" ht="13.5" customHeight="1">
       <c r="A44" s="7"/>
-      <c r="B44" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="C44" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="D44" s="25" t="s">
+      <c r="B44" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="D44" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E44" s="25"/>
-      <c r="F44" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="G44" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="H44" s="24" t="s">
-        <v>96</v>
+      <c r="E44" s="27"/>
+      <c r="F44" s="27"/>
+      <c r="G44" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="H44" s="26" t="s">
+        <v>98</v>
       </c>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
@@ -2578,22 +2580,22 @@
     </row>
     <row r="45" ht="13.5" customHeight="1">
       <c r="A45" s="7"/>
-      <c r="B45" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="C45" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D45" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="E45" s="25"/>
-      <c r="F45" s="25"/>
-      <c r="G45" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="H45" s="24" t="s">
-        <v>98</v>
+      <c r="B45" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="C45" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D45" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="E45" s="27"/>
+      <c r="F45" s="27"/>
+      <c r="G45" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="H45" s="26">
+        <v>3.12345678E8</v>
       </c>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
@@ -2616,22 +2618,22 @@
     </row>
     <row r="46" ht="13.5" customHeight="1">
       <c r="A46" s="7"/>
-      <c r="B46" s="24" t="s">
-        <v>99</v>
-      </c>
-      <c r="C46" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="D46" s="25" t="s">
+      <c r="B46" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="C46" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="D46" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="E46" s="25"/>
-      <c r="F46" s="25"/>
-      <c r="G46" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="H46" s="24">
-        <v>3.12345678E8</v>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="H46" s="26">
+        <v>9.01234567E8</v>
       </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
@@ -2654,22 +2656,24 @@
     </row>
     <row r="47" ht="13.5" customHeight="1">
       <c r="A47" s="7"/>
-      <c r="B47" s="24" t="s">
-        <v>101</v>
-      </c>
-      <c r="C47" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D47" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="E47" s="25"/>
-      <c r="F47" s="25"/>
-      <c r="G47" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="H47" s="24">
-        <v>9.01234567E8</v>
+      <c r="B47" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C47" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D47" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="F47" s="27"/>
+      <c r="G47" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="H47" s="26" t="s">
+        <v>47</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
@@ -2692,24 +2696,22 @@
     </row>
     <row r="48" ht="13.5" customHeight="1">
       <c r="A48" s="7"/>
-      <c r="B48" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="C48" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D48" s="25" t="s">
+      <c r="B48" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C48" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="D48" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E48" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="F48" s="25"/>
-      <c r="G48" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="H48" s="24" t="s">
-        <v>47</v>
+      <c r="E48" s="27"/>
+      <c r="F48" s="27"/>
+      <c r="G48" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="H48" s="28">
+        <v>46288.33333333334</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
@@ -2732,22 +2734,24 @@
     </row>
     <row r="49" ht="13.5" customHeight="1">
       <c r="A49" s="7"/>
-      <c r="B49" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="C49" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="D49" s="25" t="s">
+      <c r="B49" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="C49" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E49" s="25"/>
-      <c r="F49" s="25"/>
-      <c r="G49" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="H49" s="26">
-        <v>46288.33333333334</v>
+      <c r="E49" s="27"/>
+      <c r="F49" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="G49" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="H49" s="27">
+        <v>101.0</v>
       </c>
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
@@ -2770,24 +2774,22 @@
     </row>
     <row r="50" ht="13.5" customHeight="1">
       <c r="A50" s="7"/>
-      <c r="B50" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="C50" s="25" t="s">
-        <v>11</v>
-      </c>
-      <c r="D50" s="25" t="s">
+      <c r="B50" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="C50" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="D50" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E50" s="25"/>
-      <c r="F50" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="G50" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="H50" s="25">
-        <v>101.0</v>
+      <c r="E50" s="27"/>
+      <c r="F50" s="27"/>
+      <c r="G50" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="H50" s="28">
+        <v>46288.375</v>
       </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
@@ -2809,23 +2811,25 @@
       <c r="Z50" s="2"/>
     </row>
     <row r="51" ht="13.5" customHeight="1">
-      <c r="A51" s="7"/>
-      <c r="B51" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="C51" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="D51" s="25" t="s">
+      <c r="A51" s="9"/>
+      <c r="B51" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="C51" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="E51" s="25"/>
-      <c r="F51" s="25"/>
-      <c r="G51" s="25" t="s">
-        <v>55</v>
-      </c>
-      <c r="H51" s="26">
-        <v>46288.375</v>
+      <c r="E51" s="27"/>
+      <c r="F51" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="G51" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="H51" s="27">
+        <v>101.0</v>
       </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
@@ -2847,25 +2851,27 @@
       <c r="Z51" s="2"/>
     </row>
     <row r="52" ht="13.5" customHeight="1">
-      <c r="A52" s="9"/>
-      <c r="B52" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="C52" s="25" t="s">
+      <c r="A52" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="B52" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="C52" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="D52" s="25" t="s">
+      <c r="D52" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E52" s="25"/>
-      <c r="F52" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="G52" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="H52" s="25">
-        <v>101.0</v>
+      <c r="E52" s="31"/>
+      <c r="F52" s="31" t="s">
+        <v>72</v>
+      </c>
+      <c r="G52" s="31" t="s">
+        <v>105</v>
+      </c>
+      <c r="H52" s="31">
+        <v>1001.0</v>
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
@@ -2887,27 +2893,25 @@
       <c r="Z52" s="2"/>
     </row>
     <row r="53" ht="13.5" customHeight="1">
-      <c r="A53" s="27" t="s">
-        <v>104</v>
-      </c>
-      <c r="B53" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="C53" s="29" t="s">
+      <c r="A53" s="7"/>
+      <c r="B53" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C53" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="D53" s="29" t="s">
+      <c r="D53" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E53" s="29"/>
-      <c r="F53" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="G53" s="29" t="s">
-        <v>106</v>
-      </c>
-      <c r="H53" s="29">
-        <v>1001.0</v>
+      <c r="E53" s="31"/>
+      <c r="F53" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="G53" s="31" t="s">
+        <v>108</v>
+      </c>
+      <c r="H53" s="31">
+        <v>5001.0</v>
       </c>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
@@ -2930,24 +2934,22 @@
     </row>
     <row r="54" ht="13.5" customHeight="1">
       <c r="A54" s="7"/>
-      <c r="B54" s="28" t="s">
-        <v>107</v>
-      </c>
-      <c r="C54" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D54" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E54" s="29"/>
-      <c r="F54" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="G54" s="29" t="s">
+      <c r="B54" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="29">
-        <v>5001.0</v>
+      <c r="C54" s="31" t="s">
+        <v>29</v>
+      </c>
+      <c r="D54" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="E54" s="31"/>
+      <c r="F54" s="31"/>
+      <c r="G54" s="31" t="s">
+        <v>110</v>
+      </c>
+      <c r="H54" s="30" t="s">
+        <v>111</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
@@ -2970,22 +2972,24 @@
     </row>
     <row r="55" ht="13.5" customHeight="1">
       <c r="A55" s="7"/>
-      <c r="B55" s="28" t="s">
-        <v>110</v>
-      </c>
-      <c r="C55" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="D55" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="E55" s="29"/>
-      <c r="F55" s="29"/>
-      <c r="G55" s="29" t="s">
-        <v>111</v>
-      </c>
-      <c r="H55" s="28" t="s">
+      <c r="B55" s="32" t="s">
         <v>112</v>
+      </c>
+      <c r="C55" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="D55" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" s="32" t="b">
+        <v>0</v>
+      </c>
+      <c r="F55" s="32"/>
+      <c r="G55" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="H55" s="32" t="b">
+        <v>1</v>
       </c>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
@@ -3009,23 +3013,21 @@
     <row r="56" ht="13.5" customHeight="1">
       <c r="A56" s="7"/>
       <c r="B56" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="C56" s="30" t="s">
-        <v>39</v>
-      </c>
-      <c r="D56" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="C56" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D56" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E56" s="30" t="b">
-        <v>0</v>
-      </c>
+      <c r="E56" s="31"/>
       <c r="F56" s="31"/>
-      <c r="G56" s="30" t="s">
-        <v>114</v>
-      </c>
-      <c r="H56" s="30" t="b">
-        <v>1</v>
+      <c r="G56" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="H56" s="33">
+        <v>46288.33333333334</v>
       </c>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
@@ -3048,22 +3050,24 @@
     </row>
     <row r="57" ht="13.5" customHeight="1">
       <c r="A57" s="7"/>
-      <c r="B57" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="C57" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="D57" s="29" t="s">
+      <c r="B57" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="C57" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E57" s="29"/>
-      <c r="F57" s="29"/>
-      <c r="G57" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="H57" s="32">
-        <v>46288.33333333334</v>
+      <c r="E57" s="31"/>
+      <c r="F57" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="G57" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="H57" s="31">
+        <v>101.0</v>
       </c>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
@@ -3086,24 +3090,22 @@
     </row>
     <row r="58" ht="13.5" customHeight="1">
       <c r="A58" s="7"/>
-      <c r="B58" s="28" t="s">
-        <v>51</v>
-      </c>
-      <c r="C58" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D58" s="29" t="s">
+      <c r="B58" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="C58" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D58" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E58" s="29"/>
-      <c r="F58" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="G58" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="H58" s="29">
-        <v>101.0</v>
+      <c r="E58" s="31"/>
+      <c r="F58" s="31"/>
+      <c r="G58" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="H58" s="33">
+        <v>46288.375</v>
       </c>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
@@ -3125,23 +3127,25 @@
       <c r="Z58" s="2"/>
     </row>
     <row r="59" ht="13.5" customHeight="1">
-      <c r="A59" s="7"/>
-      <c r="B59" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="C59" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="D59" s="29" t="s">
+      <c r="A59" s="9"/>
+      <c r="B59" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="C59" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E59" s="29"/>
-      <c r="F59" s="29"/>
-      <c r="G59" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H59" s="32">
-        <v>46288.375</v>
+      <c r="E59" s="31"/>
+      <c r="F59" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="G59" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="H59" s="31">
+        <v>101.0</v>
       </c>
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
@@ -3163,26 +3167,14 @@
       <c r="Z59" s="2"/>
     </row>
     <row r="60" ht="13.5" customHeight="1">
-      <c r="A60" s="9"/>
-      <c r="B60" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="C60" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D60" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E60" s="29"/>
-      <c r="F60" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="G60" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="H60" s="29">
-        <v>101.0</v>
-      </c>
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
@@ -29522,42 +29514,14 @@
       <c r="Y1000" s="2"/>
       <c r="Z1000" s="2"/>
     </row>
-    <row r="1001" ht="13.5" customHeight="1">
-      <c r="A1001" s="2"/>
-      <c r="B1001" s="2"/>
-      <c r="C1001" s="2"/>
-      <c r="D1001" s="2"/>
-      <c r="E1001" s="2"/>
-      <c r="F1001" s="2"/>
-      <c r="G1001" s="2"/>
-      <c r="H1001" s="2"/>
-      <c r="I1001" s="2"/>
-      <c r="J1001" s="2"/>
-      <c r="K1001" s="2"/>
-      <c r="L1001" s="2"/>
-      <c r="M1001" s="2"/>
-      <c r="N1001" s="2"/>
-      <c r="O1001" s="2"/>
-      <c r="P1001" s="2"/>
-      <c r="Q1001" s="2"/>
-      <c r="R1001" s="2"/>
-      <c r="S1001" s="2"/>
-      <c r="T1001" s="2"/>
-      <c r="U1001" s="2"/>
-      <c r="V1001" s="2"/>
-      <c r="W1001" s="2"/>
-      <c r="X1001" s="2"/>
-      <c r="Y1001" s="2"/>
-      <c r="Z1001" s="2"/>
-    </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A2:A15"/>
     <mergeCell ref="A16:A24"/>
-    <mergeCell ref="A25:A32"/>
-    <mergeCell ref="A33:A42"/>
-    <mergeCell ref="A43:A52"/>
-    <mergeCell ref="A53:A60"/>
+    <mergeCell ref="A42:A51"/>
+    <mergeCell ref="A52:A59"/>
+    <mergeCell ref="A25:A31"/>
+    <mergeCell ref="A32:A41"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>